<commit_message>
Enhance attendance record export functionality
- Added total fines calculation and summary sheet generation in the Excel export.
- Introduced a new summary sheet to display student-specific attendance data and total fines.
- Updated the Excel export format to include additional styling and improved layout for better readability.
- Implemented logic to aggregate attendance records by student, including counts for present, late, and absent statuses.
</commit_message>
<xml_diff>
--- a/data/attendance_log.xlsx
+++ b/data/attendance_log.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -537,12 +537,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>MATTHEW KARL LOUIS B. SALVOSA</t>
+          <t>test</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>22-20123</t>
+          <t>22-20000</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -561,35 +561,35 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>GJ270JNU</t>
+          <t>2YO5TJD4, 2CZAP83Z</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Dave</t>
+          <t>Dave Majait</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>22-203254</t>
+          <t>22-20002</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -608,10 +608,10 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>1</v>
@@ -624,54 +624,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>GJ270JNU</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>louis</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>22-2032543</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>BSCS</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>GJ270JNU</t>
+          <t>2YO5TJD4, 2CZAP83Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance student management features
- Updated the student detail page to include a button for resetting all data related to a student, including attendance records, manual fines, and payments.
- Introduced a new API endpoint to clear all manual fines for a student, with confirmation prompts for user actions.
- Enhanced the session management interface to allow customization of fine settings per session, including late, partial, and absent fines.
- Improved the database schema to support new fine settings and scheduled start times for sessions.
- Updated Excel export functionality to include manual fines and payments in the summary sheet for better financial tracking.
</commit_message>
<xml_diff>
--- a/data/attendance_log.xlsx
+++ b/data/attendance_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$O$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,13 +33,8 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00721c24"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -50,12 +45,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="001a1a2e"/>
         <bgColor rgb="001a1a2e"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00f8d7da"/>
-        <bgColor rgb="00f8d7da"/>
       </patternFill>
     </fill>
   </fills>
@@ -85,15 +74,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -461,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -474,7 +460,11 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,10 +515,30 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Attendance Fines (PHP)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Manual Fines (PHP)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Total Fines (PHP)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Total Paid (PHP)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Balance (PHP)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Sessions List</t>
         </is>
@@ -537,12 +547,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>JAMIL P. MANANGUITE</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>22-20000</t>
+          <t>22-01179</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -552,7 +562,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -561,35 +571,47 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J2" s="3" t="n">
-        <v>75</v>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>2YO5TJD4, 2CZAP83Z</t>
+        <v>0</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Dave Majait</t>
+          <t>MA. LHOREN A. BANAR</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>22-20002</t>
+          <t>24-10755</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -599,7 +621,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -608,28 +630,571 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>2YO5TJD4, 2CZAP83Z</t>
+      <c r="J3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>MARIA JULIA J. PALOMERAS</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>25-10258</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>ELMER A. TENORIO</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>25-10290</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ALGIN V. SABUCO</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>25-10424</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>LEO CARL C. INDINO</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>25-10489</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>FRANCINE L. DEALAGDON</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>25-10572</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>FIL JUSTIN D. BALZA</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>25-10608</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>DIANA ELIZABETH I. DELOS SANTOS</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>25-10754</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>MARK VINCE M. VILLARANTE</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>25-10810</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>NICOLE ANN SUICO</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>25-10872</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:O1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Enhance record export functionality and UI
- Added a dropdown menu for exporting records by session in the records template, improving user experience and accessibility.
- Updated the API download logic to map session IDs to session names for clearer file naming and improved data presentation.
- Refactored the Excel export headers to reflect the new session naming convention.
- Improved JavaScript functionality for toggling the export dropdown and handling user interactions.
</commit_message>
<xml_diff>
--- a/data/attendance_log.xlsx
+++ b/data/attendance_log.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,8 +33,18 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00721c24"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00856404"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -45,6 +55,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="001a1a2e"/>
         <bgColor rgb="001a1a2e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f8d7da"/>
+        <bgColor rgb="00f8d7da"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fff3cd"/>
+        <bgColor rgb="00fff3cd"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,12 +96,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -447,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -547,12 +575,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>JAMIL P. MANANGUITE</t>
+          <t>Bescoro, Jennifer I.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>22-01179</t>
+          <t>14-00521</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -562,7 +590,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -577,41 +605,41 @@
         <v>1</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" s="2" t="n">
-        <v>0</v>
+      <c r="L2" s="3" t="n">
+        <v>50</v>
       </c>
       <c r="M2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N2" s="2" t="n">
-        <v>0</v>
+      <c r="N2" s="4" t="n">
+        <v>50</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>B2BZ0J76</t>
+          <t>WCRNXP1W</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>MA. LHOREN A. BANAR</t>
+          <t>ROEY PLOI G. LOPAR</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>24-10755</t>
+          <t>17-00092</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -621,7 +649,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -639,38 +667,38 @@
         <v>0</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L3" s="2" t="n">
-        <v>0</v>
+      <c r="L3" s="3" t="n">
+        <v>25</v>
       </c>
       <c r="M3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N3" s="2" t="n">
-        <v>0</v>
+      <c r="N3" s="4" t="n">
+        <v>25</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>B2BZ0J76</t>
+          <t>WCRNXP1W</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MARIA JULIA J. PALOMERAS</t>
+          <t>Rosales, Ma. Patricia J.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>25-10258</t>
+          <t>21-00454</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -680,7 +708,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -695,41 +723,41 @@
         <v>1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L4" s="2" t="n">
-        <v>0</v>
+      <c r="L4" s="3" t="n">
+        <v>50</v>
       </c>
       <c r="M4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N4" s="2" t="n">
-        <v>0</v>
+      <c r="N4" s="4" t="n">
+        <v>50</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>B2BZ0J76</t>
+          <t>WCRNXP1W</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ELMER A. TENORIO</t>
+          <t>Garcio, Eduard Jess J.</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>25-10290</t>
+          <t>22-00996</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -739,7 +767,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -754,41 +782,41 @@
         <v>1</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="2" t="n">
-        <v>0</v>
+      <c r="L5" s="3" t="n">
+        <v>50</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="2" t="n">
-        <v>0</v>
+      <c r="N5" s="4" t="n">
+        <v>50</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>B2BZ0J76</t>
+          <t>WCRNXP1W</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ALGIN V. SABUCO</t>
+          <t>JAMIL P. MANANGUITE</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>25-10424</t>
+          <t>22-01179</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -842,12 +870,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>LEO CARL C. INDINO</t>
+          <t>Aler, Vianney Jeff M.</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>25-10489</t>
+          <t>23-10453</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -857,7 +885,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -872,41 +900,41 @@
         <v>1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="2" t="n">
-        <v>0</v>
+      <c r="L7" s="3" t="n">
+        <v>50</v>
       </c>
       <c r="M7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N7" s="2" t="n">
-        <v>0</v>
+      <c r="N7" s="4" t="n">
+        <v>50</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>B2BZ0J76</t>
+          <t>WCRNXP1W</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>FRANCINE L. DEALAGDON</t>
+          <t>JALBEN T. TAMAYO</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>25-10572</t>
+          <t>24-10135</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -916,7 +944,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -953,19 +981,19 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>B2BZ0J76</t>
+          <t>WCRNXP1W</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>FIL JUSTIN D. BALZA</t>
+          <t>RENATO JR. P. MONTERON</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>25-10608</t>
+          <t>24-10145</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -975,7 +1003,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -993,38 +1021,38 @@
         <v>0</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="2" t="n">
-        <v>0</v>
+      <c r="L9" s="3" t="n">
+        <v>25</v>
       </c>
       <c r="M9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N9" s="2" t="n">
-        <v>0</v>
+      <c r="N9" s="4" t="n">
+        <v>25</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>B2BZ0J76</t>
+          <t>WCRNXP1W</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>DIANA ELIZABETH I. DELOS SANTOS</t>
+          <t>CHARLES KENT C. TALA</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>25-10754</t>
+          <t>24-10146</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1034,7 +1062,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1071,19 +1099,19 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>B2BZ0J76</t>
+          <t>WCRNXP1W</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>MARK VINCE M. VILLARANTE</t>
+          <t>Carin, Carl E.</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>25-10810</t>
+          <t>24-10159</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1093,7 +1121,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1108,86 +1136,1384 @@
         <v>1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="2" t="n">
-        <v>0</v>
+      <c r="L11" s="3" t="n">
+        <v>50</v>
       </c>
       <c r="M11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N11" s="2" t="n">
-        <v>0</v>
+      <c r="N11" s="4" t="n">
+        <v>50</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>B2BZ0J76</t>
+          <t>WCRNXP1W</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>JUSTIN PAUL A. BELANO</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>24-10161</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Laguna, Mark A.</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>24-10204</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>KENNETH C. PONDANG</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>24-10231</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>JHON PAUL B. MAHAYAG</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>24-10242</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>RAUL BRENT S. COLLAMAT</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>24-10260</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Layong, John Wayne D.</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>24-10274</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Torrefiel, Khel Renz L.</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>24-10275</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Sumile, Yushi R.</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>24-10367</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>JUSTINE V. PIAMONTE</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>24-10509</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Albelda, Kristoff Jimre Q.</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>24-10530</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Durmiendo, Drizzle S.</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>24-10565</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Lucenesio, Rhea M.</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>24-10592</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Ecraela, Pamela R.</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>24-10689</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>WCRNXP1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>MA. LHOREN A. BANAR</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>24-10755</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>MARIA JULIA J. PALOMERAS</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>25-10258</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>ELMER A. TENORIO</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>25-10290</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>ALGIN V. SABUCO</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>25-10424</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>LEO CARL C. INDINO</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>25-10489</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>FRANCINE L. DEALAGDON</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>25-10572</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>FIL JUSTIN D. BALZA</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>25-10608</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>DIANA ELIZABETH I. DELOS SANTOS</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>25-10754</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>MARK VINCE M. VILLARANTE</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>25-10810</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>B2BZ0J76</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t>NICOLE ANN SUICO</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>25-10872</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>BSCS</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>BSCS</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>B2BZ0J76</t>
         </is>

</xml_diff>